<commit_message>
Enforce monthly cross-counter relationships
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/收银员与柜组关系导入模板.xlsx
+++ b/templates/收银员与柜组关系导入模板.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\A 百分点科技\02  TS250003-中免\00 中免需求对接\20260624 店长看板需求\北京机场店-收银分析\收银员与柜组关系维护\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15395DA4-2E5F-4A2F-8F91-07ED342289F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B5326D1-F9FF-4E69-A8A6-539400E4192D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" xr2:uid="{766B619C-AB03-41BF-B1AC-CF44B7707A70}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="48">
   <si>
     <t>月份</t>
   </si>
@@ -175,6 +175,12 @@
   <si>
     <t>跨柜组</t>
   </si>
+  <si>
+    <t>跨柜组规则</t>
+  </si>
+  <si>
+    <t>跨柜组仅在同一月份、同一工号关联多个不同柜组时有意义；不同月份的柜组关系不参与跨柜组核对。</t>
+  </si>
 </sst>
 </file>
 
@@ -249,7 +255,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -275,6 +281,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5139,7 +5148,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38664CD7-8F57-4B7E-B319-593D797D0674}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.59765625" customWidth="1"/>
@@ -5216,6 +5225,14 @@
       </c>
       <c r="B9" s="8" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="27.75" x14ac:dyDescent="0.4">
+      <c r="A10" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>